<commit_message>
feat(hw01): update TC05 to PASS boundary clamp, sync 20 user defects, regenerate artifacts and package 23120372_HW01_AI_100.zip
</commit_message>
<xml_diff>
--- a/Test_Cases_and_Checklist.xlsx
+++ b/Test_Cases_and_Checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test Summary Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -785,37 +785,37 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Keypad Controller</t>
+          <t>Dimmer Boundary</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Evaluate switch debounce and race-condition tolerance under high-frequency key actuations</t>
+          <t>Verify upper boundary clamping when Brightness (+) is pressed at maximum (100%)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Lamp is powered ON in Warm Yellow mode</t>
+          <t>Lamp is powered ON at Level 10 (100% max brightness)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1. Actuate Mode button rapidly 10 times within 1.5 seconds (&lt; 150ms per press). 2. Observe cycle progression and controller latency.</t>
+          <t>1. Set lamp to Level 10 (100% max brightness). 2. Press Brightness (+) button 3 additional times. 3. Inspect optical output and controller state.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Controller filters contact bounce cleanly, registers each pulse, and stops on expected mode (10 mod 3 = step 2: Cool White).</t>
+          <t>Luminance remains clamped at 100% without flickering, restarting, or overflowing controller register.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Controller missed 3 pulses due to poor debounce timing; light momentarily froze before switching to Warm+White.</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Luminance remained stable at 100%; no unwanted state transitions occurred.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>DEF-04</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -842,27 +842,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Verify upper boundary clamping when Brightness (+) is pressed at maximum (100%)</t>
+          <t>Verify lower boundary clamping when Brightness (-) is pressed at minimum (~10%)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Lamp is powered ON at Level 10 (100% max brightness)</t>
+          <t>Lamp is powered ON at Level 1 (lowest brightness)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1. Press Brightness (+) button 3 additional times. 2. Inspect optical output and controller state.</t>
+          <t>1. Press Brightness (-) button 3 additional times. 2. Inspect optical output and controller state.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Luminance remains clamped at 100% without flickering, restarting, or overflowing controller register.</t>
+          <t>Luminance remains clamped at lowest step without turning completely OFF.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Luminance remained stable at 100%; no unwanted state transitions.</t>
+          <t>Luminance remained stable at lowest step; lamp did not extinguish.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -889,37 +889,37 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dimmer Boundary</t>
+          <t>Keypad Controller</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Verify lower boundary clamping when Brightness (-) is pressed at minimum (~10%)</t>
+          <t>Evaluate switch debounce and race-condition tolerance under high-frequency key actuations</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Lamp is powered ON at Level 1 (lowest brightness)</t>
+          <t>Lamp is powered ON in Warm Yellow mode</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1. Press Brightness (-) button 3 additional times. 2. Inspect optical output and controller state.</t>
+          <t>1. Actuate Mode button rapidly 10 times within 1.5 seconds (&lt; 150ms per press). 2. Observe cycle progression and controller latency.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Luminance remains clamped at lowest step without turning completely OFF.</t>
+          <t>Controller filters contact bounce cleanly, registers each pulse, and stops on expected mode (10 mod 3 = step 2: Cool White).</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Luminance remained stable at lowest step; lamp did not turn off.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Controller missed 3 pulses due to poor debounce timing; light momentarily froze before switching to Mixed mode.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>DEF-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update real Google Drive demo video links in report, csv, xlsx, pdf and zip
</commit_message>
<xml_diff>
--- a/Test_Cases_and_Checklist.xlsx
+++ b/Test_Cases_and_Checklist.xlsx
@@ -513,7 +513,7 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="39" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -612,7 +612,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>https://youtu.be/dummy_tc01_unlisted</t>
+          <t>https://drive.google.com/file/d/1AqzEp-ahpQb8BXGxQtEYIK0z55KglzjW/view?usp=drive_link</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://youtu.be/dummy_tc02_unlisted</t>
+          <t>https://drive.google.com/file/d/1SdJ5tnL_fClKkOi-Wxa4iglX7SsH-MTS/view?usp=drive_link</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://youtu.be/dummy_tc03_unlisted</t>
+          <t>https://drive.google.com/file/d/1PYIPAXF51-eJAg62AJ44-gmAANnmq0yS/view?usp=drive_link</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://youtu.be/dummy_tc04_unlisted</t>
+          <t>https://drive.google.com/file/d/1GvF7-akn0I3OsxeWWId2PdWFkCvqdspF/view?usp=drive_link</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://youtu.be/dummy_tc05_unlisted</t>
+          <t>https://drive.google.com/file/d/1esOgORvNQ2H1uxuzIsKlqoRIeqZG5oZd/view?usp=drive_link</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">

</xml_diff>